<commit_message>
final: promote r09 (pass_rate 0.8725) over r03 (0.855)
r09 is the full 400 run at 95b2de5: submit recalculates and refuses on
unconfirmed error cells, and the instructions stop over-filling answer
ranges and spell out how labels, display strings and numbers are written
(issue #16). Against r03: 24 tasks gained, 17 lost, 4 of the 33 never-pass
tasks fixed. cell_accuracy 0.8123 (r03 0.8273), pass_rate_sheet_level 0.824
(0.808), pass_rate_cell_level 0.8945 (0.8764).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CatrdSNKb3R1J9vS9deMkH
</commit_message>
<xml_diff>
--- a/outputs/10452.xlsx
+++ b/outputs/10452.xlsx
@@ -247,52 +247,56 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="3" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="3" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="3" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -551,117 +555,117 @@
   <dimension ref="A2:G15"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="69.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="29.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="4.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="69.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="29.66"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="6"/>
+      <c r="E4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="5"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="1"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>